<commit_message>
Refresh Shiny app data 2026-08-10 18:07
</commit_message>
<xml_diff>
--- a/Seymour_etal_2017/Seymour_etal_2017_TableS1_snapshot.xlsx
+++ b/Seymour_etal_2017/Seymour_etal_2017_TableS1_snapshot.xlsx
@@ -3942,13 +3942,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{474F97E6-8F81-4096-B473-F8029C3198DF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F89F99E-600F-4C65-A66D-E3B595B2F95B}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{668A7EE0-8A32-4049-B470-FE5A9C2820E3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{837B915C-DCB8-4085-BF4A-716D86ADAFE4}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{682F4353-6B3D-48F2-BD10-7C0B84ED275C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45AD9BB6-30B5-4847-B57D-8E513B43CB53}"/>
 </file>
</xml_diff>

<commit_message>
Refresh Shiny app data 2026-08-18 16:49
</commit_message>
<xml_diff>
--- a/Seymour_etal_2017/Seymour_etal_2017_TableS1_snapshot.xlsx
+++ b/Seymour_etal_2017/Seymour_etal_2017_TableS1_snapshot.xlsx
@@ -3942,13 +3942,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3271EC90-9850-4BA4-9776-19E7AC5FEE08}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85A75A14-F980-4FA4-A770-B73FE9013EED}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2F0921C4-2524-45DF-8550-AFD10405BD20}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{184D64C0-C3EE-4DEE-BD57-36D16C1EBF3A}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D0EB1840-88A4-4CD9-8DE2-8FC4ACE8FB10}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5491CE31-6B17-4525-A924-166A1F2A38AF}"/>
 </file>
</xml_diff>